<commit_message>
feat: regenerate diagrams and CRC cards for refined model
</commit_message>
<xml_diff>
--- a/docs/crc.xlsx
+++ b/docs/crc.xlsx
@@ -12,10 +12,12 @@
     <sheet name="Bidder" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Moderator" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ITradingRules" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Auction" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Lot" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Bid" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="AcquiringService" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="IAcquiringService" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="AuctionStatus" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Auction" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Lot" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Bid" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AcquiringService" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,18 +37,24 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -68,13 +76,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -442,11 +450,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,50 +463,177 @@
           <t>Учасник аукціону (AuctionParticipant)</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Зберігати participantId і displayName</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Seller</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Ідентифікувати роль учасника</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>— (базовий клас для ролей)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Надавати спільну роль учасника</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Надавати відображуване ім’я</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ставка (Bid)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>обов’язки класу</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>з ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Зберігати суму ставки</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Bidder</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Moderator</t>
-        </is>
-      </c>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Зберігати час подання і учасника</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Сервіс еквайрингу (AcquiringService)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>обов’язки класу</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>з ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Симулювати списання коштів</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Bidder</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Повідомляти про результат списання</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -517,8 +652,8 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,50 +662,55 @@
           <t>Продавець (Seller)</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Створювати лот з описом і стартовою ціною</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Створювати лот</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Подавати аукціон на модерацію або знімати його</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Подавати аукціон на модерацію</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Auction</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Moderator</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Знімати аукціон</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -586,11 +726,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -599,48 +739,45 @@
           <t>Учасник торгів (Bidder)</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Подавати ставки в дозволений час</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Подавати ставки за правилами</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Auction</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Переглядати власні прийняті ставки</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Переглядати власні ставки</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Bid</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>ITradingRules</t>
         </is>
       </c>
     </row>
@@ -658,11 +795,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -671,50 +808,43 @@
           <t>Модератор (Moderator)</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Перевіряти відповідність лоту правилам</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Перевіряти аукціон</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Auction</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Схвалювати або відхиляти аукціон</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Lot</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>ITradingRules</t>
-        </is>
-      </c>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -730,11 +860,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -743,50 +873,31 @@
           <t>Правила торгів (ITradingRules)</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Визначати, чи дозволена операція для лоту</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Seller</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Bidder</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Moderator</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Перевіряти можливість виконання операції</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
@@ -806,89 +917,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Аукціон (Auction)</t>
-        </is>
-      </c>
+          <t>Сервіс еквайрингу (IAcquiringService)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Керувати життєвим циклом торгів</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Seller</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Перевіряти та приймати ставки</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Moderator</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Визначати переможця і finalPrice</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Приймати запит на списання коштів</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Bidder</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Lot</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>AcquiringService</t>
         </is>
       </c>
     </row>
@@ -909,52 +977,53 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Лот (Lot)</t>
-        </is>
-      </c>
+          <t>Стан аукціону (AuctionStatus)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Зберігати опис і стартову ціну</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Повертати українську назву стану</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Auction</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Композиційно зберігати прийняті ставки</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Представляти сім визначених станів</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -965,6 +1034,95 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Аукціон (Auction)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>обов’язки класу</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>з ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Керувати життєвим циклом</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Перевіряти та приймати ставки</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Bidder</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Завершувати торги й визначати переможця</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>IAcquiringService</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Фіксувати підсумкову ціну</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -973,120 +1131,65 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ставка (Bid)</t>
-        </is>
-      </c>
+          <t>Лот (Lot)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>обов’язки класу</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>з ким співпрацює</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Зберігати amount, submittedAt і bidder</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Зберігати опис і стартову ціну</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Створювати та зберігати ставки</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Bidder</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Lot</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Auction</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Сервіс еквайрингу (AcquiringService)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>обов’язки класу</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>з ким співпрацює</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Симулювати списання після визначення переможця</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Auction</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Не виконувати реальних мережевих платежів</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Bidder</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Повертати найвищу ставку</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
fix: align diagrams with refined model
</commit_message>
<xml_diff>
--- a/docs/crc.xlsx
+++ b/docs/crc.xlsx
@@ -463,7 +463,6 @@
           <t>Учасник аукціону (AuctionParticipant)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -528,7 +527,6 @@
           <t>Ставка (Bid)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -597,7 +595,6 @@
           <t>Сервіс еквайрингу (AcquiringService)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -662,7 +659,6 @@
           <t>Продавець (Seller)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -739,7 +735,6 @@
           <t>Учасник торгів (Bidder)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -808,7 +803,6 @@
           <t>Модератор (Moderator)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -873,7 +867,6 @@
           <t>Правила торгів (ITradingRules)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -930,7 +923,6 @@
           <t>Сервіс еквайрингу (IAcquiringService)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -987,7 +979,6 @@
           <t>Стан аукціону (AuctionStatus)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -1052,7 +1043,6 @@
           <t>Аукціон (Auction)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -1112,7 +1102,11 @@
           <t>Фіксувати підсумкову ціну</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>AuctionStatus</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1141,7 +1135,6 @@
           <t>Лот (Lot)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>

</xml_diff>